<commit_message>
7ths and Borrowed Chords
Implemented 7th Chords as well as Borrowed Chords (Look at the 'Ending,' 'Blues,' and 'Funky' chord progressions)
Working on melody generation for an accompaniment.
</commit_message>
<xml_diff>
--- a/MidiPyGenStatus.xlsx
+++ b/MidiPyGenStatus.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="84">
   <si>
     <t>Date</t>
   </si>
@@ -253,6 +253,24 @@
   </si>
   <si>
     <t>Add Percussion</t>
+  </si>
+  <si>
+    <t>ERROR: QUINTET DOESN’T WORK! ENDS UP WITH DIATONIC OF 0 FOR EXTRA INSTRUMENT</t>
+  </si>
+  <si>
+    <t>Feature additions</t>
+  </si>
+  <si>
+    <t>In Work</t>
+  </si>
+  <si>
+    <t>Quintet error is fixed</t>
+  </si>
+  <si>
+    <t>Borrowed Chords and Seventh Chords</t>
+  </si>
+  <si>
+    <t>Melody generation using motif and periods</t>
   </si>
 </sst>
 </file>
@@ -572,7 +590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -613,6 +631,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="1" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -652,8 +673,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1009,13 +1029,13 @@
       <c r="I3" s="21"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="45">
+      <c r="A4" s="48">
         <v>43095</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="49" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="23" t="s">
@@ -1028,9 +1048,9 @@
       <c r="I4" s="25"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="45"/>
-      <c r="B5" s="41"/>
-      <c r="C5" s="46"/>
+      <c r="A5" s="48"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="49"/>
       <c r="D5" s="26" t="s">
         <v>10</v>
       </c>
@@ -1043,14 +1063,14 @@
       <c r="I5" s="27"/>
     </row>
     <row r="6" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="45"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="43" t="s">
+      <c r="A6" s="48"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
       <c r="G6" s="8" t="s">
         <v>15</v>
       </c>
@@ -1058,14 +1078,14 @@
       <c r="I6" s="27"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="45"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="43" t="s">
+      <c r="A7" s="48"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
       <c r="G7" s="8" t="s">
         <v>19</v>
       </c>
@@ -1073,14 +1093,14 @@
       <c r="I7" s="27"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="45"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="43" t="s">
+      <c r="A8" s="48"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="47"/>
       <c r="G8" s="8" t="s">
         <v>20</v>
       </c>
@@ -1088,9 +1108,9 @@
       <c r="I8" s="27"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="45"/>
-      <c r="B9" s="41"/>
-      <c r="C9" s="46"/>
+      <c r="A9" s="48"/>
+      <c r="B9" s="44"/>
+      <c r="C9" s="49"/>
       <c r="D9" s="26" t="s">
         <v>14</v>
       </c>
@@ -1101,9 +1121,9 @@
       <c r="I9" s="27"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="45"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="46"/>
+      <c r="A10" s="48"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="49"/>
       <c r="D10" s="28" t="s">
         <v>16</v>
       </c>
@@ -1114,9 +1134,9 @@
       <c r="I10" s="27"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="45"/>
-      <c r="B11" s="42"/>
-      <c r="C11" s="46"/>
+      <c r="A11" s="48"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="49"/>
       <c r="D11" s="29" t="s">
         <v>17</v>
       </c>
@@ -1127,13 +1147,13 @@
       <c r="I11" s="31"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="34">
+      <c r="A12" s="37">
         <v>43097</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="40" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="23" t="s">
@@ -1146,9 +1166,9 @@
       <c r="I12" s="25"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="35"/>
-      <c r="B13" s="41"/>
-      <c r="C13" s="38"/>
+      <c r="A13" s="38"/>
+      <c r="B13" s="44"/>
+      <c r="C13" s="41"/>
       <c r="D13" s="26" t="s">
         <v>22</v>
       </c>
@@ -1161,9 +1181,9 @@
       <c r="I13" s="27"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="35"/>
-      <c r="B14" s="41"/>
-      <c r="C14" s="38"/>
+      <c r="A14" s="38"/>
+      <c r="B14" s="44"/>
+      <c r="C14" s="41"/>
       <c r="D14" s="28" t="s">
         <v>23</v>
       </c>
@@ -1176,9 +1196,9 @@
       <c r="I14" s="27"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="35"/>
-      <c r="B15" s="41"/>
-      <c r="C15" s="38"/>
+      <c r="A15" s="38"/>
+      <c r="B15" s="44"/>
+      <c r="C15" s="41"/>
       <c r="D15" s="28" t="s">
         <v>30</v>
       </c>
@@ -1191,9 +1211,9 @@
       <c r="I15" s="27"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="35"/>
-      <c r="B16" s="41"/>
-      <c r="C16" s="38"/>
+      <c r="A16" s="38"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="28" t="s">
         <v>25</v>
       </c>
@@ -1204,9 +1224,9 @@
       <c r="I16" s="27"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="35"/>
-      <c r="B17" s="41"/>
-      <c r="C17" s="38"/>
+      <c r="A17" s="38"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="41"/>
       <c r="D17" s="28" t="s">
         <v>26</v>
       </c>
@@ -1217,9 +1237,9 @@
       <c r="I17" s="27"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="35"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="38"/>
+      <c r="A18" s="38"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="41"/>
       <c r="D18" s="28" t="s">
         <v>29</v>
       </c>
@@ -1230,9 +1250,9 @@
       <c r="I18" s="27"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="35"/>
-      <c r="B19" s="41"/>
-      <c r="C19" s="38"/>
+      <c r="A19" s="38"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="41"/>
       <c r="D19" s="28"/>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
@@ -1241,9 +1261,9 @@
       <c r="I19" s="27"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="35"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="38"/>
+      <c r="A20" s="38"/>
+      <c r="B20" s="44"/>
+      <c r="C20" s="41"/>
       <c r="D20" s="26" t="s">
         <v>10</v>
       </c>
@@ -1256,9 +1276,9 @@
       <c r="I20" s="27"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="35"/>
-      <c r="B21" s="41"/>
-      <c r="C21" s="38"/>
+      <c r="A21" s="38"/>
+      <c r="B21" s="44"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="28" t="s">
         <v>31</v>
       </c>
@@ -1271,9 +1291,9 @@
       <c r="I21" s="27"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="35"/>
-      <c r="B22" s="41"/>
-      <c r="C22" s="38"/>
+      <c r="A22" s="38"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="41"/>
       <c r="D22" s="28" t="s">
         <v>24</v>
       </c>
@@ -1286,9 +1306,9 @@
       <c r="I22" s="27"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="35"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="38"/>
+      <c r="A23" s="38"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="41"/>
       <c r="D23" s="1" t="s">
         <v>34</v>
       </c>
@@ -1301,9 +1321,9 @@
       <c r="I23" s="27"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="36"/>
-      <c r="B24" s="42"/>
-      <c r="C24" s="39"/>
+      <c r="A24" s="39"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="42"/>
       <c r="D24" s="29" t="s">
         <v>35</v>
       </c>
@@ -1316,13 +1336,13 @@
       <c r="I24" s="31"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="45">
+      <c r="A25" s="48">
         <v>43100</v>
       </c>
-      <c r="B25" s="45" t="s">
+      <c r="B25" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="C25" s="46" t="s">
+      <c r="C25" s="49" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="23" t="s">
@@ -1335,9 +1355,9 @@
       <c r="I25" s="25"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="45"/>
-      <c r="B26" s="45"/>
-      <c r="C26" s="46"/>
+      <c r="A26" s="48"/>
+      <c r="B26" s="48"/>
+      <c r="C26" s="49"/>
       <c r="D26" s="26" t="s">
         <v>22</v>
       </c>
@@ -1350,9 +1370,9 @@
       <c r="I26" s="27"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="45"/>
-      <c r="B27" s="45"/>
-      <c r="C27" s="46"/>
+      <c r="A27" s="48"/>
+      <c r="B27" s="48"/>
+      <c r="C27" s="49"/>
       <c r="D27" s="28" t="s">
         <v>39</v>
       </c>
@@ -1365,9 +1385,9 @@
       <c r="I27" s="27"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="45"/>
-      <c r="B28" s="45"/>
-      <c r="C28" s="46"/>
+      <c r="A28" s="48"/>
+      <c r="B28" s="48"/>
+      <c r="C28" s="49"/>
       <c r="D28" s="28" t="s">
         <v>40</v>
       </c>
@@ -1380,9 +1400,9 @@
       <c r="I28" s="27"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="45"/>
-      <c r="B29" s="45"/>
-      <c r="C29" s="46"/>
+      <c r="A29" s="48"/>
+      <c r="B29" s="48"/>
+      <c r="C29" s="49"/>
       <c r="D29" s="26" t="s">
         <v>50</v>
       </c>
@@ -1395,9 +1415,9 @@
       <c r="I29" s="27"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="45"/>
-      <c r="B30" s="45"/>
-      <c r="C30" s="46"/>
+      <c r="A30" s="48"/>
+      <c r="B30" s="48"/>
+      <c r="C30" s="49"/>
       <c r="D30" s="28" t="s">
         <v>51</v>
       </c>
@@ -1410,9 +1430,9 @@
       <c r="I30" s="27"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="45"/>
-      <c r="B31" s="45"/>
-      <c r="C31" s="46"/>
+      <c r="A31" s="48"/>
+      <c r="B31" s="48"/>
+      <c r="C31" s="49"/>
       <c r="D31" s="28" t="s">
         <v>52</v>
       </c>
@@ -1425,9 +1445,9 @@
       <c r="I31" s="27"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="45"/>
-      <c r="B32" s="45"/>
-      <c r="C32" s="46"/>
+      <c r="A32" s="48"/>
+      <c r="B32" s="48"/>
+      <c r="C32" s="49"/>
       <c r="D32" s="28" t="s">
         <v>53</v>
       </c>
@@ -1442,9 +1462,9 @@
       <c r="I32" s="27"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="45"/>
-      <c r="B33" s="45"/>
-      <c r="C33" s="46"/>
+      <c r="A33" s="48"/>
+      <c r="B33" s="48"/>
+      <c r="C33" s="49"/>
       <c r="D33" s="28" t="s">
         <v>55</v>
       </c>
@@ -1457,9 +1477,9 @@
       <c r="I33" s="27"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="45"/>
-      <c r="B34" s="45"/>
-      <c r="C34" s="46"/>
+      <c r="A34" s="48"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="49"/>
       <c r="D34" s="28" t="s">
         <v>56</v>
       </c>
@@ -1472,9 +1492,9 @@
       <c r="I34" s="27"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="45"/>
-      <c r="B35" s="45"/>
-      <c r="C35" s="46"/>
+      <c r="A35" s="48"/>
+      <c r="B35" s="48"/>
+      <c r="C35" s="49"/>
       <c r="D35" s="28" t="s">
         <v>58</v>
       </c>
@@ -1487,9 +1507,9 @@
       <c r="I35" s="27"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="45"/>
-      <c r="B36" s="45"/>
-      <c r="C36" s="46"/>
+      <c r="A36" s="48"/>
+      <c r="B36" s="48"/>
+      <c r="C36" s="49"/>
       <c r="D36" s="28" t="s">
         <v>57</v>
       </c>
@@ -1504,9 +1524,9 @@
       <c r="I36" s="27"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="45"/>
-      <c r="B37" s="45"/>
-      <c r="C37" s="46"/>
+      <c r="A37" s="48"/>
+      <c r="B37" s="48"/>
+      <c r="C37" s="49"/>
       <c r="D37" s="28" t="s">
         <v>59</v>
       </c>
@@ -1526,9 +1546,9 @@
       <c r="I37" s="27"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="45"/>
-      <c r="B38" s="45"/>
-      <c r="C38" s="46"/>
+      <c r="A38" s="48"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="49"/>
       <c r="D38" s="28" t="s">
         <v>60</v>
       </c>
@@ -1545,9 +1565,9 @@
       <c r="I38" s="27"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="45"/>
-      <c r="B39" s="45"/>
-      <c r="C39" s="46"/>
+      <c r="A39" s="48"/>
+      <c r="B39" s="48"/>
+      <c r="C39" s="49"/>
       <c r="D39" s="28" t="s">
         <v>61</v>
       </c>
@@ -1564,9 +1584,9 @@
       <c r="I39" s="27"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="45"/>
-      <c r="B40" s="45"/>
-      <c r="C40" s="46"/>
+      <c r="A40" s="48"/>
+      <c r="B40" s="48"/>
+      <c r="C40" s="49"/>
       <c r="D40" s="28" t="s">
         <v>57</v>
       </c>
@@ -1581,9 +1601,9 @@
       <c r="I40" s="27"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="45"/>
-      <c r="B41" s="45"/>
-      <c r="C41" s="46"/>
+      <c r="A41" s="48"/>
+      <c r="B41" s="48"/>
+      <c r="C41" s="49"/>
       <c r="D41" s="28" t="s">
         <v>64</v>
       </c>
@@ -1600,9 +1620,9 @@
       <c r="I41" s="27"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="45"/>
-      <c r="B42" s="45"/>
-      <c r="C42" s="46"/>
+      <c r="A42" s="48"/>
+      <c r="B42" s="48"/>
+      <c r="C42" s="49"/>
       <c r="D42" s="28" t="s">
         <v>68</v>
       </c>
@@ -1619,9 +1639,9 @@
       <c r="I42" s="27"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="45"/>
-      <c r="B43" s="45"/>
-      <c r="C43" s="46"/>
+      <c r="A43" s="48"/>
+      <c r="B43" s="48"/>
+      <c r="C43" s="49"/>
       <c r="D43" s="29" t="s">
         <v>67</v>
       </c>
@@ -1638,19 +1658,19 @@
       <c r="I43" s="31"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="40">
+      <c r="A44" s="43">
         <v>43104</v>
       </c>
-      <c r="B44" s="40" t="s">
+      <c r="B44" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C44" s="37" t="s">
+      <c r="C44" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="D44" s="47" t="s">
+      <c r="D44" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="E44" s="48" t="s">
+      <c r="E44" s="35" t="s">
         <v>74</v>
       </c>
       <c r="F44" s="24"/>
@@ -1659,9 +1679,9 @@
       <c r="I44" s="25"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" s="41"/>
-      <c r="B45" s="41"/>
-      <c r="C45" s="38"/>
+      <c r="A45" s="44"/>
+      <c r="B45" s="44"/>
+      <c r="C45" s="41"/>
       <c r="D45" s="28" t="s">
         <v>69</v>
       </c>
@@ -1672,9 +1692,9 @@
       <c r="I45" s="27"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="41"/>
-      <c r="B46" s="41"/>
-      <c r="C46" s="38"/>
+      <c r="A46" s="44"/>
+      <c r="B46" s="44"/>
+      <c r="C46" s="41"/>
       <c r="D46" s="28" t="s">
         <v>70</v>
       </c>
@@ -1685,9 +1705,9 @@
       <c r="I46" s="27"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" s="41"/>
-      <c r="B47" s="41"/>
-      <c r="C47" s="38"/>
+      <c r="A47" s="44"/>
+      <c r="B47" s="44"/>
+      <c r="C47" s="41"/>
       <c r="D47" s="26" t="s">
         <v>71</v>
       </c>
@@ -1698,9 +1718,9 @@
       <c r="I47" s="27"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A48" s="41"/>
-      <c r="B48" s="41"/>
-      <c r="C48" s="38"/>
+      <c r="A48" s="44"/>
+      <c r="B48" s="44"/>
+      <c r="C48" s="41"/>
       <c r="D48" s="28" t="s">
         <v>72</v>
       </c>
@@ -1711,9 +1731,9 @@
       <c r="I48" s="27"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="41"/>
-      <c r="B49" s="41"/>
-      <c r="C49" s="38"/>
+      <c r="A49" s="44"/>
+      <c r="B49" s="44"/>
+      <c r="C49" s="41"/>
       <c r="D49" s="28" t="s">
         <v>76</v>
       </c>
@@ -1724,9 +1744,9 @@
       <c r="I49" s="27"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A50" s="41"/>
-      <c r="B50" s="41"/>
-      <c r="C50" s="38"/>
+      <c r="A50" s="44"/>
+      <c r="B50" s="44"/>
+      <c r="C50" s="41"/>
       <c r="D50" s="28"/>
       <c r="E50" s="8" t="s">
         <v>75</v>
@@ -1737,9 +1757,9 @@
       <c r="I50" s="27"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" s="41"/>
-      <c r="B51" s="41"/>
-      <c r="C51" s="38"/>
+      <c r="A51" s="44"/>
+      <c r="B51" s="44"/>
+      <c r="C51" s="41"/>
       <c r="D51" s="28" t="s">
         <v>73</v>
       </c>
@@ -1750,67 +1770,86 @@
       <c r="I51" s="27"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" s="42"/>
-      <c r="B52" s="42"/>
-      <c r="C52" s="39"/>
+      <c r="A52" s="45"/>
+      <c r="B52" s="45"/>
+      <c r="C52" s="42"/>
       <c r="D52" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="E52" s="30"/>
+      <c r="E52" s="36" t="s">
+        <v>78</v>
+      </c>
       <c r="F52" s="30"/>
       <c r="G52" s="30"/>
       <c r="H52" s="30"/>
       <c r="I52" s="31"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A53" s="32"/>
-      <c r="B53" s="32"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="8"/>
-      <c r="F53" s="8"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="8"/>
-      <c r="I53" s="9"/>
+      <c r="A53" s="48">
+        <v>43107</v>
+      </c>
+      <c r="B53" s="48" t="s">
+        <v>2</v>
+      </c>
+      <c r="C53" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="D53" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="E53" s="24"/>
+      <c r="F53" s="24"/>
+      <c r="G53" s="50" t="s">
+        <v>80</v>
+      </c>
+      <c r="H53" s="24"/>
+      <c r="I53" s="25"/>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A54" s="32"/>
-      <c r="B54" s="32"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="8"/>
+      <c r="A54" s="48"/>
+      <c r="B54" s="48"/>
+      <c r="C54" s="49"/>
+      <c r="D54" s="28" t="s">
+        <v>81</v>
+      </c>
       <c r="E54" s="8"/>
       <c r="F54" s="8"/>
-      <c r="G54" s="8"/>
+      <c r="G54" s="8" t="s">
+        <v>83</v>
+      </c>
       <c r="H54" s="8"/>
-      <c r="I54" s="9"/>
+      <c r="I54" s="27"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" s="32"/>
-      <c r="B55" s="32"/>
-      <c r="C55" s="7"/>
-      <c r="D55" s="8"/>
+      <c r="A55" s="48"/>
+      <c r="B55" s="48"/>
+      <c r="C55" s="49"/>
+      <c r="D55" s="26" t="s">
+        <v>79</v>
+      </c>
       <c r="E55" s="8"/>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
-      <c r="I55" s="9"/>
+      <c r="I55" s="27"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="32"/>
-      <c r="B56" s="32"/>
-      <c r="C56" s="7"/>
-      <c r="D56" s="8"/>
-      <c r="E56" s="8"/>
-      <c r="F56" s="8"/>
-      <c r="G56" s="8"/>
-      <c r="H56" s="8"/>
-      <c r="I56" s="9"/>
+      <c r="A56" s="48"/>
+      <c r="B56" s="48"/>
+      <c r="C56" s="49"/>
+      <c r="D56" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="E56" s="30"/>
+      <c r="F56" s="30"/>
+      <c r="G56" s="30"/>
+      <c r="H56" s="30"/>
+      <c r="I56" s="31"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="32"/>
       <c r="B57" s="32"/>
       <c r="C57" s="7"/>
-      <c r="D57" s="8"/>
       <c r="E57" s="8"/>
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
@@ -2841,7 +2880,10 @@
       <c r="I150" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="18">
+    <mergeCell ref="C53:C56"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="A53:A56"/>
     <mergeCell ref="A25:A43"/>
     <mergeCell ref="B25:B43"/>
     <mergeCell ref="C25:C43"/>

</xml_diff>